<commit_message>
auto: add 01-Projects (1), add 03-Memory (1), modify 01-Projects (3), modify 03-Memory (2)
</commit_message>
<xml_diff>
--- a/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
+++ b/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="1-卡片信息" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="999" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="403">
   <si>
     <t>信用卡卡片总览 — 韩伟</t>
   </si>
@@ -1425,10 +1425,6 @@
   </si>
   <si>
     <t>和卡1  账单日不一样</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>建行 需线下</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
@@ -2100,6 +2096,9 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="3" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2128,9 +2127,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="3" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2617,15 +2613,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="95" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
+      <c r="B1" s="96"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
+      <c r="G1" s="96"/>
     </row>
     <row r="2" spans="1:8" ht="24.95" customHeight="1">
       <c r="A2" s="1" t="s">
@@ -2666,10 +2662,10 @@
       <c r="D3" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="110">
+      <c r="E3" s="94">
         <v>0</v>
       </c>
-      <c r="F3" s="110">
+      <c r="F3" s="94">
         <v>0</v>
       </c>
       <c r="G3" s="57" t="s">
@@ -3052,12 +3048,12 @@
       </c>
     </row>
     <row r="19" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A19" s="100" t="s">
+      <c r="A19" s="101" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="98"/>
-      <c r="C19" s="98"/>
-      <c r="D19" s="99"/>
+      <c r="B19" s="99"/>
+      <c r="C19" s="99"/>
+      <c r="D19" s="100"/>
       <c r="E19" s="3">
         <f>SUM(E3:E18)</f>
         <v>831000</v>
@@ -3070,26 +3066,26 @@
       <c r="H19" s="26"/>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A21" s="96" t="s">
+      <c r="A21" s="97" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="95"/>
-      <c r="C21" s="95"/>
-      <c r="D21" s="95"/>
-      <c r="E21" s="95"/>
-      <c r="F21" s="95"/>
-      <c r="G21" s="95"/>
+      <c r="B21" s="96"/>
+      <c r="C21" s="96"/>
+      <c r="D21" s="96"/>
+      <c r="E21" s="96"/>
+      <c r="F21" s="96"/>
+      <c r="G21" s="96"/>
     </row>
     <row r="24" spans="1:8" ht="21" customHeight="1">
-      <c r="A24" s="94" t="s">
+      <c r="A24" s="95" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="95"/>
-      <c r="C24" s="95"/>
-      <c r="D24" s="95"/>
-      <c r="E24" s="95"/>
-      <c r="F24" s="95"/>
-      <c r="G24" s="95"/>
+      <c r="B24" s="96"/>
+      <c r="C24" s="96"/>
+      <c r="D24" s="96"/>
+      <c r="E24" s="96"/>
+      <c r="F24" s="96"/>
+      <c r="G24" s="96"/>
     </row>
     <row r="25" spans="1:8" ht="21" customHeight="1">
       <c r="A25" s="38" t="s">
@@ -3376,12 +3372,12 @@
       <c r="H37" s="53"/>
     </row>
     <row r="38" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A38" s="97" t="s">
+      <c r="A38" s="98" t="s">
         <v>73</v>
       </c>
-      <c r="B38" s="98"/>
-      <c r="C38" s="98"/>
-      <c r="D38" s="99"/>
+      <c r="B38" s="99"/>
+      <c r="C38" s="99"/>
+      <c r="D38" s="100"/>
       <c r="E38" s="41">
         <f>SUM(E26:E37)</f>
         <v>44000</v>
@@ -3428,28 +3424,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="95" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="95"/>
+      <c r="B1" s="96"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
+      <c r="G1" s="96"/>
+      <c r="H1" s="96"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1">
-      <c r="A3" s="102" t="s">
+      <c r="A3" s="103" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="98"/>
-      <c r="C3" s="98"/>
-      <c r="D3" s="98"/>
-      <c r="E3" s="98"/>
-      <c r="F3" s="98"/>
-      <c r="G3" s="98"/>
-      <c r="H3" s="99"/>
+      <c r="B3" s="99"/>
+      <c r="C3" s="99"/>
+      <c r="D3" s="99"/>
+      <c r="E3" s="99"/>
+      <c r="F3" s="99"/>
+      <c r="G3" s="99"/>
+      <c r="H3" s="100"/>
       <c r="I3" s="24"/>
     </row>
     <row r="4" spans="1:9" ht="33" customHeight="1">
@@ -3609,16 +3605,16 @@
       <c r="I9" s="13"/>
     </row>
     <row r="10" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A10" s="102" t="s">
+      <c r="A10" s="103" t="s">
         <v>94</v>
       </c>
-      <c r="B10" s="98"/>
-      <c r="C10" s="98"/>
-      <c r="D10" s="98"/>
-      <c r="E10" s="98"/>
-      <c r="F10" s="98"/>
-      <c r="G10" s="98"/>
-      <c r="H10" s="99"/>
+      <c r="B10" s="99"/>
+      <c r="C10" s="99"/>
+      <c r="D10" s="99"/>
+      <c r="E10" s="99"/>
+      <c r="F10" s="99"/>
+      <c r="G10" s="99"/>
+      <c r="H10" s="100"/>
       <c r="I10" s="24"/>
     </row>
     <row r="11" spans="1:9" ht="16.5" customHeight="1">
@@ -3851,16 +3847,16 @@
       <c r="I19" s="13"/>
     </row>
     <row r="20" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A20" s="102" t="s">
+      <c r="A20" s="103" t="s">
         <v>109</v>
       </c>
-      <c r="B20" s="98"/>
-      <c r="C20" s="98"/>
-      <c r="D20" s="98"/>
-      <c r="E20" s="98"/>
-      <c r="F20" s="98"/>
-      <c r="G20" s="98"/>
-      <c r="H20" s="99"/>
+      <c r="B20" s="99"/>
+      <c r="C20" s="99"/>
+      <c r="D20" s="99"/>
+      <c r="E20" s="99"/>
+      <c r="F20" s="99"/>
+      <c r="G20" s="99"/>
+      <c r="H20" s="100"/>
       <c r="I20" s="24"/>
     </row>
     <row r="21" spans="1:9" ht="16.5" customHeight="1">
@@ -3985,16 +3981,16 @@
       <c r="I25" s="13"/>
     </row>
     <row r="26" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A26" s="102" t="s">
+      <c r="A26" s="103" t="s">
         <v>117</v>
       </c>
-      <c r="B26" s="98"/>
-      <c r="C26" s="98"/>
-      <c r="D26" s="98"/>
-      <c r="E26" s="98"/>
-      <c r="F26" s="98"/>
-      <c r="G26" s="98"/>
-      <c r="H26" s="99"/>
+      <c r="B26" s="99"/>
+      <c r="C26" s="99"/>
+      <c r="D26" s="99"/>
+      <c r="E26" s="99"/>
+      <c r="F26" s="99"/>
+      <c r="G26" s="99"/>
+      <c r="H26" s="100"/>
       <c r="I26" s="24"/>
     </row>
     <row r="27" spans="1:9" ht="16.5" customHeight="1">
@@ -4110,16 +4106,16 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A33" s="101" t="s">
+      <c r="A33" s="102" t="s">
         <v>133</v>
       </c>
-      <c r="B33" s="95"/>
-      <c r="C33" s="95"/>
-      <c r="D33" s="95"/>
-      <c r="E33" s="95"/>
-      <c r="F33" s="95"/>
-      <c r="G33" s="95"/>
-      <c r="H33" s="95"/>
+      <c r="B33" s="96"/>
+      <c r="C33" s="96"/>
+      <c r="D33" s="96"/>
+      <c r="E33" s="96"/>
+      <c r="F33" s="96"/>
+      <c r="G33" s="96"/>
+      <c r="H33" s="96"/>
     </row>
     <row r="36" spans="1:9" ht="14.25" customHeight="1">
       <c r="A36" s="36" t="s">
@@ -4528,24 +4524,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="95" t="s">
         <v>392</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
+      <c r="B1" s="96"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="96" t="s">
+      <c r="A2" s="97" t="s">
         <v>152</v>
       </c>
-      <c r="B2" s="95"/>
-      <c r="C2" s="95"/>
-      <c r="D2" s="95"/>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
+      <c r="B2" s="96"/>
+      <c r="C2" s="96"/>
+      <c r="D2" s="96"/>
+      <c r="E2" s="96"/>
+      <c r="F2" s="96"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -4996,7 +4992,7 @@
         <v>385</v>
       </c>
       <c r="B27" s="69" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C27" s="69" t="s">
         <v>19</v>
@@ -5074,34 +5070,34 @@
       <c r="F30" s="72"/>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A31" s="96" t="s">
+      <c r="A31" s="97" t="s">
         <v>153</v>
       </c>
-      <c r="B31" s="95"/>
-      <c r="C31" s="95"/>
-      <c r="D31" s="95"/>
-      <c r="E31" s="95"/>
-      <c r="F31" s="95"/>
+      <c r="B31" s="96"/>
+      <c r="C31" s="96"/>
+      <c r="D31" s="96"/>
+      <c r="E31" s="96"/>
+      <c r="F31" s="96"/>
     </row>
     <row r="32" spans="1:8" s="89" customFormat="1" ht="30" customHeight="1">
-      <c r="A32" s="94" t="s">
+      <c r="A32" s="95" t="s">
         <v>393</v>
       </c>
-      <c r="B32" s="95"/>
-      <c r="C32" s="95"/>
-      <c r="D32" s="95"/>
-      <c r="E32" s="95"/>
-      <c r="F32" s="95"/>
+      <c r="B32" s="96"/>
+      <c r="C32" s="96"/>
+      <c r="D32" s="96"/>
+      <c r="E32" s="96"/>
+      <c r="F32" s="96"/>
     </row>
     <row r="33" spans="1:8" s="89" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A33" s="96" t="s">
+      <c r="A33" s="97" t="s">
         <v>152</v>
       </c>
-      <c r="B33" s="95"/>
-      <c r="C33" s="95"/>
-      <c r="D33" s="95"/>
-      <c r="E33" s="95"/>
-      <c r="F33" s="95"/>
+      <c r="B33" s="96"/>
+      <c r="C33" s="96"/>
+      <c r="D33" s="96"/>
+      <c r="E33" s="96"/>
+      <c r="F33" s="96"/>
     </row>
     <row r="34" spans="1:8" s="89" customFormat="1" ht="15" customHeight="1">
       <c r="A34" s="1" t="s">
@@ -5137,7 +5133,7 @@
         <v>100000</v>
       </c>
       <c r="E35" s="69">
-        <v>100000</v>
+        <v>88888</v>
       </c>
       <c r="F35" s="70" t="s">
         <v>399</v>
@@ -5156,9 +5152,7 @@
     </row>
     <row r="37" spans="1:8" s="89" customFormat="1" ht="16.5" customHeight="1">
       <c r="A37" s="69"/>
-      <c r="B37" s="8" t="s">
-        <v>402</v>
-      </c>
+      <c r="B37" s="8"/>
       <c r="C37" s="8"/>
       <c r="D37" s="69"/>
       <c r="E37" s="8"/>
@@ -5422,7 +5416,7 @@
       </c>
       <c r="E54" s="72">
         <f>SUM(E12:E53)</f>
-        <v>1486300</v>
+        <v>1475188</v>
       </c>
       <c r="F54" s="72"/>
     </row>
@@ -5502,28 +5496,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="95" t="s">
         <v>156</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="95"/>
+      <c r="B1" s="96"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
+      <c r="G1" s="96"/>
+      <c r="H1" s="96"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="103" t="s">
+      <c r="A3" s="104" t="s">
         <v>157</v>
       </c>
-      <c r="B3" s="95"/>
-      <c r="C3" s="95"/>
-      <c r="D3" s="95"/>
-      <c r="E3" s="95"/>
-      <c r="F3" s="95"/>
-      <c r="G3" s="95"/>
-      <c r="H3" s="95"/>
+      <c r="B3" s="96"/>
+      <c r="C3" s="96"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
+      <c r="F3" s="96"/>
+      <c r="G3" s="96"/>
+      <c r="H3" s="96"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -5838,10 +5832,10 @@
       </c>
     </row>
     <row r="16" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A16" s="104" t="s">
+      <c r="A16" s="105" t="s">
         <v>197</v>
       </c>
-      <c r="B16" s="105"/>
+      <c r="B16" s="106"/>
       <c r="C16" s="8">
         <f>SUM(C5:C15)</f>
         <v>35</v>
@@ -5854,21 +5848,21 @@
         <f>SUM(E5:E15)</f>
         <v>35</v>
       </c>
-      <c r="F16" s="104" t="s">
+      <c r="F16" s="105" t="s">
         <v>198</v>
       </c>
-      <c r="G16" s="105"/>
+      <c r="G16" s="106"/>
       <c r="H16" s="21"/>
     </row>
     <row r="17" spans="1:8" ht="15" customHeight="1">
-      <c r="A17" s="95"/>
-      <c r="B17" s="95"/>
-      <c r="C17" s="95"/>
-      <c r="D17" s="95"/>
-      <c r="E17" s="95"/>
-      <c r="F17" s="95"/>
-      <c r="G17" s="95"/>
-      <c r="H17" s="95"/>
+      <c r="A17" s="96"/>
+      <c r="B17" s="96"/>
+      <c r="C17" s="96"/>
+      <c r="D17" s="96"/>
+      <c r="E17" s="96"/>
+      <c r="F17" s="96"/>
+      <c r="G17" s="96"/>
+      <c r="H17" s="96"/>
     </row>
     <row r="18" spans="1:8" ht="15" customHeight="1">
       <c r="A18" s="33" t="s">
@@ -6265,25 +6259,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="95" t="s">
         <v>222</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="95"/>
+      <c r="B1" s="96"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
+      <c r="G1" s="96"/>
+      <c r="H1" s="96"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="103" t="s">
+      <c r="A3" s="104" t="s">
         <v>223</v>
       </c>
-      <c r="B3" s="95"/>
-      <c r="C3" s="95"/>
-      <c r="D3" s="95"/>
-      <c r="E3" s="95"/>
+      <c r="B3" s="96"/>
+      <c r="C3" s="96"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -6371,16 +6365,16 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
-      <c r="A11" s="103" t="s">
+      <c r="A11" s="104" t="s">
         <v>243</v>
       </c>
-      <c r="B11" s="95"/>
-      <c r="C11" s="95"/>
-      <c r="D11" s="95"/>
-      <c r="E11" s="95"/>
-      <c r="F11" s="95"/>
-      <c r="G11" s="95"/>
-      <c r="H11" s="95"/>
+      <c r="B11" s="96"/>
+      <c r="C11" s="96"/>
+      <c r="D11" s="96"/>
+      <c r="E11" s="96"/>
+      <c r="F11" s="96"/>
+      <c r="G11" s="96"/>
+      <c r="H11" s="96"/>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
       <c r="A12" s="1" t="s">
@@ -6536,24 +6530,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="95" t="s">
         <v>250</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
+      <c r="B1" s="96"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1">
-      <c r="A3" s="103" t="s">
+      <c r="A3" s="104" t="s">
         <v>251</v>
       </c>
-      <c r="B3" s="95"/>
-      <c r="C3" s="95"/>
-      <c r="D3" s="95"/>
-      <c r="E3" s="95"/>
-      <c r="F3" s="95"/>
+      <c r="B3" s="96"/>
+      <c r="C3" s="96"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
+      <c r="F3" s="96"/>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1">
       <c r="A4" s="5" t="s">
@@ -6636,10 +6630,10 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A8" s="108" t="s">
+      <c r="A8" s="109" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="99"/>
+      <c r="B8" s="100"/>
       <c r="C8" s="35">
         <v>500</v>
       </c>
@@ -6674,18 +6668,18 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1">
-      <c r="A10" s="106"/>
-      <c r="B10" s="98"/>
-      <c r="C10" s="98"/>
-      <c r="D10" s="98"/>
-      <c r="E10" s="98"/>
-      <c r="F10" s="99"/>
+      <c r="A10" s="107"/>
+      <c r="B10" s="99"/>
+      <c r="C10" s="99"/>
+      <c r="D10" s="99"/>
+      <c r="E10" s="99"/>
+      <c r="F10" s="100"/>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1">
-      <c r="A11" s="104" t="s">
+      <c r="A11" s="105" t="s">
         <v>197</v>
       </c>
-      <c r="B11" s="99"/>
+      <c r="B11" s="100"/>
       <c r="C11" s="34">
         <f>SUM(C5:C9)</f>
         <v>4180</v>
@@ -6746,14 +6740,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="15" customHeight="1">
-      <c r="A17" s="107" t="s">
+      <c r="A17" s="108" t="s">
         <v>265</v>
       </c>
-      <c r="B17" s="98"/>
-      <c r="C17" s="98"/>
-      <c r="D17" s="98"/>
-      <c r="E17" s="98"/>
-      <c r="F17" s="99"/>
+      <c r="B17" s="99"/>
+      <c r="C17" s="99"/>
+      <c r="D17" s="99"/>
+      <c r="E17" s="99"/>
+      <c r="F17" s="100"/>
     </row>
     <row r="18" spans="1:6" ht="15" customHeight="1">
       <c r="A18" s="11" t="s">
@@ -6804,14 +6798,14 @@
       </c>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A23" s="107" t="s">
+      <c r="A23" s="108" t="s">
         <v>163</v>
       </c>
-      <c r="B23" s="98"/>
-      <c r="C23" s="98"/>
-      <c r="D23" s="98"/>
-      <c r="E23" s="98"/>
-      <c r="F23" s="99"/>
+      <c r="B23" s="99"/>
+      <c r="C23" s="99"/>
+      <c r="D23" s="99"/>
+      <c r="E23" s="99"/>
+      <c r="F23" s="100"/>
     </row>
     <row r="24" spans="1:6" ht="16.5" customHeight="1">
       <c r="A24" s="8" t="s">
@@ -6983,28 +6977,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="95" t="s">
         <v>281</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="95"/>
+      <c r="B1" s="96"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
+      <c r="G1" s="96"/>
+      <c r="H1" s="96"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="96" t="s">
+      <c r="A2" s="97" t="s">
         <v>282</v>
       </c>
-      <c r="B2" s="95"/>
-      <c r="C2" s="95"/>
-      <c r="D2" s="95"/>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="95"/>
-      <c r="H2" s="95"/>
+      <c r="B2" s="96"/>
+      <c r="C2" s="96"/>
+      <c r="D2" s="96"/>
+      <c r="E2" s="96"/>
+      <c r="F2" s="96"/>
+      <c r="G2" s="96"/>
+      <c r="H2" s="96"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -7381,14 +7375,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="109" t="s">
+      <c r="A1" s="110" t="s">
         <v>295</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
+      <c r="B1" s="96"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
     </row>
     <row r="2" spans="1:6" ht="24.95" customHeight="1">
       <c r="A2" s="9" t="s">

</xml_diff>

<commit_message>
auto: add 01-Projects (2), modify (root) (1), modify 01-Projects (5)
</commit_message>
<xml_diff>
--- a/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
+++ b/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
@@ -25,20 +25,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1-卡片信息'!$A$2:$G$19</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 

</xml_diff>

<commit_message>
auto: add 01-Projects (1), delete 01-Projects (1), modify 01-Projects (3)
</commit_message>
<xml_diff>
--- a/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
+++ b/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
@@ -25,7 +25,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1-卡片信息'!$A$2:$G$19</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -1411,11 +1410,11 @@
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
-    <t>和卡1  账单日不一样</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
     <t>农行1(少刷)</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>和卡1账单日不一样</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
@@ -4979,7 +4978,7 @@
         <v>385</v>
       </c>
       <c r="B27" s="69" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C27" s="69" t="s">
         <v>19</v>
@@ -5181,7 +5180,7 @@
     </row>
     <row r="40" spans="1:8" s="91" customFormat="1" ht="32.25" customHeight="1">
       <c r="A40" s="69" t="s">
-        <v>318</v>
+        <v>385</v>
       </c>
       <c r="B40" s="69" t="s">
         <v>386</v>
@@ -5201,7 +5200,7 @@
         <v>351</v>
       </c>
       <c r="H40" s="92" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="14.25">

</xml_diff>